<commit_message>
Record GET-proven Crosslink Success rows on the 9/16 sheet.
Live headers 10101–10105 on batch 715 now have Select Receipts, Fees
id 11 (not PPV), and in-gate PPV. Outlook Entered in AI. invent=false.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-16-crosslink.xlsx
+++ b/runs/AP-run-2026-09-16-crosslink.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -49,11 +49,6 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -67,7 +62,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -76,9 +71,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -574,7 +566,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 3). Header PO set. Select Receipts-equivalent posted on the invoice record; do not type Add Item. Select Receipts: 1 receipt(s) matched by single open receipt on PO. Selected receipts: 23924 on PO 59087. Attach status=attached. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set. Select Receipts 23924 8@25.0 on PO 59087. Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -636,14 +628,14 @@
       <c r="E3" s="2" t="n">
         <v>830.54</v>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>HOLD (receipt): no open receipt qty matches invoice qty 4 (will not take first-open / second-open-on-po). Create KIMCO header and attach PDF; do not claim Success. HOLD: no open receipt qty matches invoice qty 4 (will not take first-open / second-open-on-po). Unmatched PO(s): 59038. Select Receipts per PO; do not skip a PO silently. Header created (id 10102). Attach status=attached. Select Receipts=held-unfinished. Outlook Entered with issues (not Entered in AI). Flag status=entered-with-issues.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set. Select Receipts 23605 3@193.94; 23794 1@193.94 on PO 59038. Fees=Packaging/Shop Supplies Recovery 8.22 (Additional Charge Fees id 11, not PPV). PPV=46.56. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -676,7 +668,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
@@ -705,14 +697,14 @@
       <c r="E4" s="2" t="n">
         <v>1174.02</v>
       </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>HOLD (receipt): no open receipt qty matches invoice qty 5 (will not take first-open / second-open-on-po). Create KIMCO header and attach PDF; do not claim Success. HOLD: no open receipt qty matches invoice qty 5 (will not take first-open / second-open-on-po). Unmatched PO(s): 59052. Select Receipts per PO; do not skip a PO silently. Header created (id 10103). Attach status=attached. Select Receipts=held-unfinished. Outlook Entered with issues (not Entered in AI). Flag status=entered-with-issues.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set. Select Receipts 23675 1@219.32; 23795 2@219.32; 23882 2@219.32 on PO 59052. Fees=Packaging/Shop Supplies Recovery 11.62 (Additional Charge Fees id 11, not PPV). PPV=65.80. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -745,7 +737,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
@@ -774,14 +766,14 @@
       <c r="E5" s="2" t="n">
         <v>1245.81</v>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>HOLD (receipt): no open receipt qty matches invoice qty 6 (will not take first-open / second-open-on-po). Create KIMCO header and attach PDF; do not claim Success. HOLD: no open receipt qty matches invoice qty 6 (will not take first-open / second-open-on-po). Unmatched PO(s): 59022. Select Receipts per PO; do not skip a PO silently. Header created (id 10104). Attach status=attached. Select Receipts=held-unfinished. Outlook Entered with issues (not Entered in AI). Flag status=entered-with-issues.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set. Select Receipts 23674 6@205.58 on PO 59022. Fees=Packaging/Shop Supplies Recovery 12.33 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -814,7 +806,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
@@ -843,14 +835,14 @@
       <c r="E6" s="2" t="n">
         <v>2104.11</v>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>HOLD (receipt): no open receipt qty matches invoice qty 8 (will not take first-open / second-open-on-po). Create KIMCO header and attach PDF; do not claim Success. HOLD: no open receipt qty matches invoice qty 8 (will not take first-open / second-open-on-po). Unmatched PO(s): 58902. Select Receipts per PO; do not skip a PO silently. Header created (id 10105). Attach status=attached. Select Receipts=held-unfinished. Outlook Entered with issues (not Entered in AI). Flag status=entered-with-issues.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set. Select Receipts 23229 8@193.94; 23230 2@219.32 on PO 58902. Fees=Packaging/Shop Supplies Recovery 20.83 (Additional Charge Fees id 11, not PPV). PPV=93.12. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -883,7 +875,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Enter Crosslink 28008 as 10106 and refresh the 9/16 sheet.
Only recent unflagged leftover after 10101–10105. Same-unit cover on
PO 58981, Fees 14.66, in-gate PPV 83.00. July 27557 not entered.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-16-crosslink.xlsx
+++ b/runs/AP-run-2026-09-16-crosslink.xlsx
@@ -10,7 +10,7 @@
     <sheet name="AP run" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$O$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$O$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -880,8 +880,77 @@
       </c>
       <c r="O6" s="2" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Crosslink Powder Coating</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>28008</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>58981</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>1480.62</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 3). Header PO set. Select Receipts 23472 1@219.32; 23231 4@193.94; 23471 2@193.94 on PO 58981. Fees=Packaging/Shop Supplies Recovery 14.66 (Additional Charge Fees id 11, not PPV). PPV=83.00. Attach status=attached. Finish Select Receipts selected ids=[23472, 23231, 23471] fees=already-posted ppv=already-posted. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>10106</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/16/26 (715)</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Packaging/Shop Supplies Recovery 14.66</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>83.00</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O6"/>
+  <autoFilter ref="A1:O7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>